<commit_message>
added Microhyla fissipes alignments and shrunk the Acanthosaura lepidogaster, Leiolepis, and Cyrtodactylus (spp_ND2_Irrawaddy) alignments
</commit_message>
<xml_diff>
--- a/Alignments_to_make.xlsx
+++ b/Alignments_to_make.xlsx
@@ -8,14 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/rklaback_byu_edu/Documents/KlabackaLab/Research/SEA-riverine-barrier-popgen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="866" documentId="8_{8806978C-AB6D-854E-872D-B0339ADE4273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DE49ED4-2410-884A-8A53-EFC5346B5BCE}"/>
+  <xr:revisionPtr revIDLastSave="1083" documentId="8_{8806978C-AB6D-854E-872D-B0339ADE4273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72D10017-9272-3944-A557-7DEFEE520B8F}"/>
   <bookViews>
-    <workbookView xWindow="42840" yWindow="-8620" windowWidth="25800" windowHeight="19180" xr2:uid="{A3120B5E-B713-6F49-8845-F185AE497150}"/>
+    <workbookView xWindow="57260" yWindow="-8620" windowWidth="11280" windowHeight="19180" xr2:uid="{A3120B5E-B713-6F49-8845-F185AE497150}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="OLE_LINK11" localSheetId="0">Sheet1!$D$221</definedName>
+    <definedName name="OLE_LINK335" localSheetId="0">Sheet1!$D$235</definedName>
+    <definedName name="OLE_LINK351" localSheetId="0">Sheet1!$D$240</definedName>
+    <definedName name="OLE_LINK363" localSheetId="0">Sheet1!$D$225</definedName>
+    <definedName name="OLE_LINK365" localSheetId="0">Sheet1!$D$229</definedName>
+    <definedName name="OLE_LINK373" localSheetId="0">Sheet1!$D$230</definedName>
+    <definedName name="OLE_LINK429" localSheetId="0">Sheet1!$D$214</definedName>
+    <definedName name="OLE_LINK431" localSheetId="0">Sheet1!$D$215</definedName>
+    <definedName name="OLE_LINK435" localSheetId="0">Sheet1!$D$214</definedName>
+    <definedName name="OLE_LINK437" localSheetId="0">Sheet1!$D$215</definedName>
+    <definedName name="OLE_LINK489" localSheetId="0">Sheet1!$D$222</definedName>
+    <definedName name="OLE_LINK599" localSheetId="0">Sheet1!$D$234</definedName>
+    <definedName name="OLE_LINK602" localSheetId="0">Sheet1!$D$236</definedName>
+    <definedName name="OLE_LINK610" localSheetId="0">Sheet1!$D$228</definedName>
+    <definedName name="OLE_LINK615" localSheetId="0">Sheet1!$D$231</definedName>
+    <definedName name="OLE_LINK633" localSheetId="0">Sheet1!$D$218</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="620">
   <si>
     <t>Species</t>
   </si>
@@ -1684,12 +1702,249 @@
   <si>
     <t>Estimate (very rough, tough to find on map. Matches map figure)</t>
   </si>
+  <si>
+    <t>Microhyla mukhlesuri</t>
+  </si>
+  <si>
+    <t>RAG2</t>
+  </si>
+  <si>
+    <t>KU882422</t>
+  </si>
+  <si>
+    <t>KU882423</t>
+  </si>
+  <si>
+    <t>KU882636</t>
+  </si>
+  <si>
+    <t>KU882637</t>
+  </si>
+  <si>
+    <t>KIZ024759</t>
+  </si>
+  <si>
+    <t>KIZ024760</t>
+  </si>
+  <si>
+    <t>KUHE34130</t>
+  </si>
+  <si>
+    <t>AB201218</t>
+  </si>
+  <si>
+    <t>KIZ024294</t>
+  </si>
+  <si>
+    <t>KIZ024295</t>
+  </si>
+  <si>
+    <t>KU882432</t>
+  </si>
+  <si>
+    <t>KU882433</t>
+  </si>
+  <si>
+    <t>KU882643</t>
+  </si>
+  <si>
+    <t>KU882644</t>
+  </si>
+  <si>
+    <t>KUHE34324</t>
+  </si>
+  <si>
+    <t>AB201221</t>
+  </si>
+  <si>
+    <t>ZISP-FN-159</t>
+  </si>
+  <si>
+    <t>KU882439</t>
+  </si>
+  <si>
+    <t>KU882649</t>
+  </si>
+  <si>
+    <t>PNKB2011.94</t>
+  </si>
+  <si>
+    <t>KU882440</t>
+  </si>
+  <si>
+    <t>Estimate (very rough, based on map)</t>
+  </si>
+  <si>
+    <t>M-E, R-S</t>
+  </si>
+  <si>
+    <t>KIZ010051</t>
+  </si>
+  <si>
+    <t>KIZ010071</t>
+  </si>
+  <si>
+    <t>KU882441</t>
+  </si>
+  <si>
+    <t>KU882442</t>
+  </si>
+  <si>
+    <t>KIZ04090</t>
+  </si>
+  <si>
+    <t>KU882358</t>
+  </si>
+  <si>
+    <t>KU882598</t>
+  </si>
+  <si>
+    <t>KU882361</t>
+  </si>
+  <si>
+    <t>KU882599</t>
+  </si>
+  <si>
+    <t>KIZ04194</t>
+  </si>
+  <si>
+    <t>KU882362</t>
+  </si>
+  <si>
+    <t>KU882600</t>
+  </si>
+  <si>
+    <t>KIZ04175</t>
+  </si>
+  <si>
+    <t>KU882364</t>
+  </si>
+  <si>
+    <t>KU882601</t>
+  </si>
+  <si>
+    <t>KIZ04163</t>
+  </si>
+  <si>
+    <t>KU882368</t>
+  </si>
+  <si>
+    <t>KU882604</t>
+  </si>
+  <si>
+    <t>KU882369</t>
+  </si>
+  <si>
+    <t>KU882605</t>
+  </si>
+  <si>
+    <t>KIZ046821</t>
+  </si>
+  <si>
+    <t>KIZ046824</t>
+  </si>
+  <si>
+    <t>Tissue ID: LC0805063</t>
+  </si>
+  <si>
+    <t>KU882376</t>
+  </si>
+  <si>
+    <t>KIZYN0705115</t>
+  </si>
+  <si>
+    <t>KIZYN0705116</t>
+  </si>
+  <si>
+    <t>KU882377</t>
+  </si>
+  <si>
+    <t>KU882609</t>
+  </si>
+  <si>
+    <t>KU882378</t>
+  </si>
+  <si>
+    <t>KU882610</t>
+  </si>
+  <si>
+    <t>KIZYN0705148</t>
+  </si>
+  <si>
+    <t>KU882382</t>
+  </si>
+  <si>
+    <t>KU882612</t>
+  </si>
+  <si>
+    <t>Microhyla fissipes</t>
+  </si>
+  <si>
+    <t>KIZ07875</t>
+  </si>
+  <si>
+    <t>KU882318</t>
+  </si>
+  <si>
+    <t>KU882567</t>
+  </si>
+  <si>
+    <t>Tissue ID: KIZYPX30172</t>
+  </si>
+  <si>
+    <t>KU882321</t>
+  </si>
+  <si>
+    <t>ROM 6618</t>
+  </si>
+  <si>
+    <t>ROM 6620</t>
+  </si>
+  <si>
+    <t>KU882322</t>
+  </si>
+  <si>
+    <t>KU882570</t>
+  </si>
+  <si>
+    <t>KU882324</t>
+  </si>
+  <si>
+    <t>KU882571</t>
+  </si>
+  <si>
+    <t>ROM 19236</t>
+  </si>
+  <si>
+    <t>ROM 19239</t>
+  </si>
+  <si>
+    <t>NAP-03351</t>
+  </si>
+  <si>
+    <t>KU882331</t>
+  </si>
+  <si>
+    <t>KU882577</t>
+  </si>
+  <si>
+    <t>KU882333</t>
+  </si>
+  <si>
+    <t>KU882578</t>
+  </si>
+  <si>
+    <t>KU882343</t>
+  </si>
+  <si>
+    <t>10.1093/cz/zow042</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1776,6 +2031,18 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1951,7 +2218,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -2004,6 +2271,43 @@
     <xf numFmtId="49" fontId="11" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2345,7 +2649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3197D522-1DFB-1F48-B517-34505A21B081}">
-  <dimension ref="A1:Q211"/>
+  <dimension ref="A1:R240"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="35.6640625" style="4" customWidth="1"/>
@@ -2353,12 +2657,12 @@
     <col min="5" max="7" width="10.83203125" style="4"/>
     <col min="8" max="8" width="14.6640625" style="4" customWidth="1"/>
     <col min="9" max="10" width="26.5" style="4" customWidth="1"/>
-    <col min="11" max="16" width="10.83203125" style="4"/>
-    <col min="17" max="17" width="14.5" style="4" customWidth="1"/>
-    <col min="18" max="16384" width="10.83203125" style="4"/>
+    <col min="11" max="17" width="10.83203125" style="4"/>
+    <col min="18" max="18" width="14.5" style="4" customWidth="1"/>
+    <col min="19" max="16384" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2390,25 +2694,28 @@
         <v>5</v>
       </c>
       <c r="L1" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A2" s="5" t="s">
         <v>12</v>
       </c>
@@ -2428,14 +2735,14 @@
       <c r="I2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="P2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="Q2" s="7" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
@@ -2455,14 +2762,14 @@
       <c r="I3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="P3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="Q3" s="7" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A4" s="5" t="s">
         <v>12</v>
       </c>
@@ -2482,14 +2789,14 @@
       <c r="I4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="P4" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="Q4" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A5" s="5" t="s">
         <v>12</v>
       </c>
@@ -2509,11 +2816,11 @@
       <c r="I5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="Q5" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A6" s="5" t="s">
         <v>12</v>
       </c>
@@ -2533,11 +2840,11 @@
       <c r="I6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="P6" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A7" s="5" t="s">
         <v>29</v>
       </c>
@@ -2557,14 +2864,14 @@
       <c r="I7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="P7" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="P7" s="7" t="s">
+      <c r="Q7" s="7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="7" customFormat="1" ht="33" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:18" s="7" customFormat="1" ht="33" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="5" t="s">
         <v>29</v>
       </c>
@@ -2584,14 +2891,14 @@
       <c r="I8" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="P8" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="P8" s="7" t="s">
+      <c r="Q8" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:17" s="12" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:18" s="12" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A9" s="11" t="s">
         <v>46</v>
       </c>
@@ -2611,11 +2918,11 @@
       <c r="I9" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="Q9" s="13" t="s">
+      <c r="R9" s="13" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A10" s="15" t="s">
         <v>67</v>
       </c>
@@ -2635,11 +2942,11 @@
       <c r="I10" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q10" s="9" t="s">
+      <c r="R10" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A11" s="15" t="s">
         <v>46</v>
       </c>
@@ -2659,11 +2966,11 @@
       <c r="I11" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q11" s="9" t="s">
+      <c r="R11" s="9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A12" s="15" t="s">
         <v>46</v>
       </c>
@@ -2683,11 +2990,11 @@
       <c r="I12" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q12" s="9" t="s">
+      <c r="R12" s="9" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="13" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A13" s="15" t="s">
         <v>46</v>
       </c>
@@ -2707,11 +3014,11 @@
       <c r="I13" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q13" s="9" t="s">
+      <c r="R13" s="9" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A14" s="15" t="s">
         <v>46</v>
       </c>
@@ -2731,11 +3038,11 @@
       <c r="I14" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q14" s="9" t="s">
+      <c r="R14" s="9" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A15" s="15" t="s">
         <v>46</v>
       </c>
@@ -2755,11 +3062,11 @@
       <c r="I15" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q15" s="9" t="s">
+      <c r="R15" s="9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A16" s="15" t="s">
         <v>46</v>
       </c>
@@ -2779,11 +3086,11 @@
       <c r="I16" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q16" s="9" t="s">
+      <c r="R16" s="9" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A17" s="15" t="s">
         <v>46</v>
       </c>
@@ -2803,11 +3110,11 @@
       <c r="I17" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q17" s="9" t="s">
+      <c r="R17" s="9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A18" s="15" t="s">
         <v>46</v>
       </c>
@@ -2827,11 +3134,11 @@
       <c r="I18" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q18" s="9" t="s">
+      <c r="R18" s="9" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A19" s="15" t="s">
         <v>69</v>
       </c>
@@ -2851,11 +3158,11 @@
       <c r="I19" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="Q19" s="9" t="s">
+      <c r="R19" s="9" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A20" s="16" t="s">
         <v>71</v>
       </c>
@@ -2875,11 +3182,11 @@
       <c r="I20" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="Q20" s="2" t="s">
+      <c r="R20" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A21" s="16" t="s">
         <v>71</v>
       </c>
@@ -2900,11 +3207,11 @@
       <c r="I21" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="Q21" s="2" t="s">
+      <c r="R21" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="22" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A22" s="16" t="s">
         <v>71</v>
       </c>
@@ -2924,11 +3231,11 @@
       <c r="I22" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="Q22" s="2" t="s">
+      <c r="R22" s="2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="23" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A23" s="16" t="s">
         <v>71</v>
       </c>
@@ -2949,11 +3256,11 @@
       <c r="I23" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="Q23" s="2" t="s">
+      <c r="R23" s="2" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A24" s="16" t="s">
         <v>71</v>
       </c>
@@ -2973,11 +3280,11 @@
       <c r="I24" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="Q24" s="2" t="s">
+      <c r="R24" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="25" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A25" s="16" t="s">
         <v>71</v>
       </c>
@@ -2999,11 +3306,11 @@
       <c r="I25" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="Q25" s="2" t="s">
+      <c r="R25" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
         <v>71</v>
       </c>
@@ -3022,11 +3329,11 @@
       <c r="I26" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="Q26" s="2" t="s">
+      <c r="R26" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A27" s="15" t="s">
         <v>90</v>
       </c>
@@ -3045,11 +3352,11 @@
       <c r="I27" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="Q27" s="9" t="s">
+      <c r="R27" s="9" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A28" s="15" t="s">
         <v>90</v>
       </c>
@@ -3068,11 +3375,11 @@
       <c r="I28" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="Q28" s="9" t="s">
+      <c r="R28" s="9" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="29" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A29" s="15" t="s">
         <v>90</v>
       </c>
@@ -3091,11 +3398,11 @@
       <c r="I29" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="Q29" s="9" t="s">
+      <c r="R29" s="9" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="30" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A30" s="15" t="s">
         <v>90</v>
       </c>
@@ -3114,11 +3421,11 @@
       <c r="I30" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="Q30" s="9" t="s">
+      <c r="R30" s="9" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="31" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A31" s="15" t="s">
         <v>90</v>
       </c>
@@ -3137,11 +3444,11 @@
       <c r="I31" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="Q31" s="9" t="s">
+      <c r="R31" s="9" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="32" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A32" s="15" t="s">
         <v>90</v>
       </c>
@@ -3160,11 +3467,11 @@
       <c r="I32" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="Q32" s="17" t="s">
+      <c r="R32" s="17" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="33" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A33" s="15" t="s">
         <v>90</v>
       </c>
@@ -3184,11 +3491,11 @@
       <c r="I33" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="Q33" s="9" t="s">
+      <c r="R33" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A34" s="15" t="s">
         <v>90</v>
       </c>
@@ -3208,11 +3515,11 @@
       <c r="I34" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="Q34" s="9" t="s">
+      <c r="R34" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="35" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A35" s="15" t="s">
         <v>90</v>
       </c>
@@ -3234,11 +3541,11 @@
       <c r="I35" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="Q35" s="9" t="s">
+      <c r="R35" s="9" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:17" s="19" customFormat="1" ht="33" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:18" s="19" customFormat="1" ht="33" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A36" s="18" t="s">
         <v>90</v>
       </c>
@@ -3257,11 +3564,11 @@
       <c r="I36" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="Q36" s="21" t="s">
+      <c r="R36" s="21" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="37" spans="1:17" s="22" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" s="22" customFormat="1" ht="17" x14ac:dyDescent="0.25">
       <c r="A37" s="22" t="s">
         <v>104</v>
       </c>
@@ -3285,15 +3592,16 @@
       <c r="K37" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="M37" s="24"/>
-      <c r="N37" s="24" t="s">
+      <c r="L37" s="24"/>
+      <c r="N37" s="24"/>
+      <c r="O37" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="O37" s="24" t="s">
+      <c r="P37" s="24" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="38" spans="1:17" s="25" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:18" s="25" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A38" s="22" t="s">
         <v>104</v>
       </c>
@@ -3316,15 +3624,16 @@
       <c r="K38" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="M38" s="24"/>
-      <c r="N38" s="24" t="s">
+      <c r="L38" s="24"/>
+      <c r="N38" s="24"/>
+      <c r="O38" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="O38" s="24" t="s">
+      <c r="P38" s="24" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="39" spans="1:17" s="25" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:18" s="25" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A39" s="22" t="s">
         <v>104</v>
       </c>
@@ -3347,15 +3656,16 @@
       <c r="K39" s="24" t="s">
         <v>116</v>
       </c>
-      <c r="M39" s="24"/>
-      <c r="N39" s="24" t="s">
+      <c r="L39" s="24"/>
+      <c r="N39" s="24"/>
+      <c r="O39" s="24" t="s">
         <v>115</v>
       </c>
-      <c r="O39" s="24" t="s">
+      <c r="P39" s="24" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:17" s="25" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:18" s="25" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A40" s="22" t="s">
         <v>104</v>
       </c>
@@ -3374,11 +3684,11 @@
       <c r="I40" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="O40" s="24" t="s">
+      <c r="P40" s="24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="41" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="22" t="s">
         <v>104</v>
       </c>
@@ -3397,11 +3707,11 @@
       <c r="I41" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="O41" s="24" t="s">
+      <c r="P41" s="24" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="42" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="22" t="s">
         <v>104</v>
       </c>
@@ -3423,11 +3733,11 @@
       <c r="I42" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="O42" s="24" t="s">
+      <c r="P42" s="24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="43" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="22" t="s">
         <v>104</v>
       </c>
@@ -3449,11 +3759,11 @@
       <c r="I43" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="O43" s="24" t="s">
+      <c r="P43" s="24" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="44" spans="1:17" s="25" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:18" s="25" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A44" s="22" t="s">
         <v>104</v>
       </c>
@@ -3475,11 +3785,11 @@
       <c r="I44" s="25" t="s">
         <v>143</v>
       </c>
-      <c r="O44" s="24" t="s">
+      <c r="P44" s="24" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="45" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="22" t="s">
         <v>104</v>
       </c>
@@ -3501,11 +3811,11 @@
       <c r="I45" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="O45" s="25" t="s">
+      <c r="P45" s="25" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="46" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="22" t="s">
         <v>104</v>
       </c>
@@ -3527,11 +3837,11 @@
       <c r="I46" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="O46" s="25" t="s">
+      <c r="P46" s="25" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="47" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="22" t="s">
         <v>104</v>
       </c>
@@ -3553,11 +3863,11 @@
       <c r="I47" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="O47" s="25" t="s">
+      <c r="P47" s="25" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="48" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="22" t="s">
         <v>104</v>
       </c>
@@ -3579,11 +3889,11 @@
       <c r="I48" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="O48" s="25" t="s">
+      <c r="P48" s="25" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="49" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="22" t="s">
         <v>104</v>
       </c>
@@ -3605,11 +3915,11 @@
       <c r="I49" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="O49" s="25" t="s">
+      <c r="P49" s="25" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="50" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="22" t="s">
         <v>104</v>
       </c>
@@ -3631,11 +3941,11 @@
       <c r="I50" s="25" t="s">
         <v>149</v>
       </c>
-      <c r="O50" s="25" t="s">
+      <c r="P50" s="25" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="51" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="22" t="s">
         <v>104</v>
       </c>
@@ -3657,11 +3967,11 @@
       <c r="I51" s="25" t="s">
         <v>142</v>
       </c>
-      <c r="O51" s="25" t="s">
+      <c r="P51" s="25" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="52" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="22" t="s">
         <v>104</v>
       </c>
@@ -3683,11 +3993,11 @@
       <c r="I52" s="25" t="s">
         <v>119</v>
       </c>
-      <c r="O52" s="25" t="s">
+      <c r="P52" s="25" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="53" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="22" t="s">
         <v>104</v>
       </c>
@@ -3709,11 +4019,11 @@
       <c r="I53" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="O53" s="25" t="s">
+      <c r="P53" s="25" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="54" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="22" t="s">
         <v>104</v>
       </c>
@@ -3727,7 +4037,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="55" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="22" t="s">
         <v>104</v>
       </c>
@@ -3749,11 +4059,11 @@
       <c r="I55" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="O55" s="25" t="s">
+      <c r="P55" s="25" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="56" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="22" t="s">
         <v>104</v>
       </c>
@@ -3776,7 +4086,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:15" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:16" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="22" t="s">
         <v>104</v>
       </c>
@@ -3798,11 +4108,11 @@
       <c r="I57" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="O57" s="25" t="s">
+      <c r="P57" s="25" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="58" spans="1:15" s="27" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" s="27" customFormat="1" ht="17" x14ac:dyDescent="0.25">
       <c r="A58" s="27" t="s">
         <v>205</v>
       </c>
@@ -3827,17 +4137,17 @@
       <c r="K58" s="27" t="s">
         <v>173</v>
       </c>
-      <c r="M58" s="27" t="s">
-        <v>171</v>
-      </c>
       <c r="N58" s="27" t="s">
         <v>171</v>
       </c>
       <c r="O58" s="27" t="s">
+        <v>171</v>
+      </c>
+      <c r="P58" s="27" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="59" spans="1:15" s="27" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" s="27" customFormat="1" ht="17" x14ac:dyDescent="0.25">
       <c r="A59" s="27" t="s">
         <v>205</v>
       </c>
@@ -3859,14 +4169,14 @@
       <c r="I59" s="27" t="s">
         <v>207</v>
       </c>
-      <c r="M59" s="27" t="s">
+      <c r="N59" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="O59" s="27" t="s">
+      <c r="P59" s="27" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="60" spans="1:15" s="27" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" s="27" customFormat="1" ht="17" x14ac:dyDescent="0.25">
       <c r="A60" s="27" t="s">
         <v>205</v>
       </c>
@@ -3891,17 +4201,17 @@
       <c r="K60" s="27" t="s">
         <v>180</v>
       </c>
-      <c r="M60" s="27" t="s">
-        <v>178</v>
-      </c>
       <c r="N60" s="27" t="s">
         <v>178</v>
       </c>
       <c r="O60" s="27" t="s">
+        <v>178</v>
+      </c>
+      <c r="P60" s="27" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="61" spans="1:15" s="27" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" s="27" customFormat="1" ht="17" x14ac:dyDescent="0.25">
       <c r="A61" s="27" t="s">
         <v>205</v>
       </c>
@@ -3926,17 +4236,17 @@
       <c r="K61" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="M61" s="27" t="s">
-        <v>181</v>
-      </c>
       <c r="N61" s="27" t="s">
         <v>181</v>
       </c>
       <c r="O61" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="P61" s="27" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="62" spans="1:15" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="27" t="s">
         <v>205</v>
       </c>
@@ -3961,17 +4271,17 @@
       <c r="K62" s="27" t="s">
         <v>191</v>
       </c>
-      <c r="M62" s="27" t="s">
+      <c r="N62" s="27" t="s">
         <v>188</v>
       </c>
-      <c r="N62" s="27" t="s">
+      <c r="O62" s="27" t="s">
         <v>189</v>
       </c>
-      <c r="O62" s="27" t="s">
+      <c r="P62" s="27" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="63" spans="1:15" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="27" t="s">
         <v>205</v>
       </c>
@@ -3993,11 +4303,11 @@
       <c r="I63" s="27" t="s">
         <v>208</v>
       </c>
-      <c r="N63" s="27" t="s">
+      <c r="O63" s="27" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="64" spans="1:15" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="27" t="s">
         <v>205</v>
       </c>
@@ -4019,14 +4329,14 @@
       <c r="I64" s="27" t="s">
         <v>208</v>
       </c>
-      <c r="N64" s="27" t="s">
+      <c r="O64" s="27" t="s">
         <v>195</v>
       </c>
-      <c r="O64" s="27" t="s">
+      <c r="P64" s="27" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="65" spans="1:15" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A65" s="27" t="s">
         <v>205</v>
       </c>
@@ -4051,17 +4361,17 @@
       <c r="K65" s="27" t="s">
         <v>200</v>
       </c>
-      <c r="M65" s="27" t="s">
-        <v>198</v>
-      </c>
       <c r="N65" s="27" t="s">
         <v>198</v>
       </c>
       <c r="O65" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="P65" s="27" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="66" spans="1:15" s="27" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="27" t="s">
         <v>205</v>
       </c>
@@ -4086,17 +4396,17 @@
       <c r="K66" s="27" t="s">
         <v>204</v>
       </c>
-      <c r="M66" s="27" t="s">
-        <v>202</v>
-      </c>
       <c r="N66" s="27" t="s">
         <v>202</v>
       </c>
       <c r="O66" s="27" t="s">
+        <v>202</v>
+      </c>
+      <c r="P66" s="27" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="67" spans="1:15" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:16" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A67" s="8" t="s">
         <v>227</v>
       </c>
@@ -4118,11 +4428,11 @@
       <c r="I67" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="N67" s="9" t="s">
+      <c r="O67" s="9" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="68" spans="1:15" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:16" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A68" s="8" t="s">
         <v>227</v>
       </c>
@@ -4144,11 +4454,11 @@
       <c r="I68" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="N68" s="9" t="s">
+      <c r="O68" s="9" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="69" spans="1:15" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:16" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A69" s="8" t="s">
         <v>227</v>
       </c>
@@ -4170,11 +4480,11 @@
       <c r="I69" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="N69" s="9" t="s">
+      <c r="O69" s="9" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="70" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A70" s="8" t="s">
         <v>227</v>
       </c>
@@ -4196,11 +4506,11 @@
       <c r="I70" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="N70" s="9" t="s">
+      <c r="O70" s="9" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="71" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="8" t="s">
         <v>227</v>
       </c>
@@ -4222,11 +4532,11 @@
       <c r="I71" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="N71" s="9" t="s">
+      <c r="O71" s="9" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="72" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A72" s="8" t="s">
         <v>227</v>
       </c>
@@ -4248,11 +4558,11 @@
       <c r="I72" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="N72" s="9" t="s">
+      <c r="O72" s="9" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="73" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="8" t="s">
         <v>227</v>
       </c>
@@ -4274,11 +4584,11 @@
       <c r="I73" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="N73" s="9" t="s">
+      <c r="O73" s="9" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="74" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="8" t="s">
         <v>227</v>
       </c>
@@ -4300,11 +4610,11 @@
       <c r="I74" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="N74" s="9" t="s">
+      <c r="O74" s="9" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="75" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A75" s="8" t="s">
         <v>227</v>
       </c>
@@ -4326,11 +4636,11 @@
       <c r="I75" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="N75" s="9" t="s">
+      <c r="O75" s="9" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="76" spans="1:15" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:16" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A76" s="31" t="s">
         <v>228</v>
       </c>
@@ -4352,11 +4662,11 @@
       <c r="I76" s="31" t="s">
         <v>207</v>
       </c>
-      <c r="N76" s="34" t="s">
+      <c r="O76" s="34" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="77" spans="1:15" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:16" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A77" s="31" t="s">
         <v>228</v>
       </c>
@@ -4378,11 +4688,11 @@
       <c r="I77" s="31" t="s">
         <v>208</v>
       </c>
-      <c r="N77" s="34" t="s">
+      <c r="O77" s="34" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="78" spans="1:15" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:16" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A78" s="31" t="s">
         <v>228</v>
       </c>
@@ -4404,11 +4714,11 @@
       <c r="I78" s="31" t="s">
         <v>207</v>
       </c>
-      <c r="N78" s="34" t="s">
+      <c r="O78" s="34" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="79" spans="1:15" s="31" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" s="31" customFormat="1" ht="17" x14ac:dyDescent="0.25">
       <c r="A79" s="31" t="s">
         <v>228</v>
       </c>
@@ -4430,11 +4740,11 @@
       <c r="I79" s="31" t="s">
         <v>208</v>
       </c>
-      <c r="N79" s="34" t="s">
+      <c r="O79" s="34" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="80" spans="1:15" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:16" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A80" s="31" t="s">
         <v>228</v>
       </c>
@@ -4456,11 +4766,11 @@
       <c r="I80" s="31" t="s">
         <v>207</v>
       </c>
-      <c r="N80" s="34" t="s">
+      <c r="O80" s="34" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="81" spans="1:17" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:18" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A81" s="31" t="s">
         <v>228</v>
       </c>
@@ -4482,11 +4792,11 @@
       <c r="I81" s="31" t="s">
         <v>207</v>
       </c>
-      <c r="N81" s="34" t="s">
+      <c r="O81" s="34" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="82" spans="1:17" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:18" s="31" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A82" s="31" t="s">
         <v>228</v>
       </c>
@@ -4508,11 +4818,11 @@
       <c r="I82" s="31" t="s">
         <v>207</v>
       </c>
-      <c r="N82" s="34" t="s">
+      <c r="O82" s="34" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="83" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A83" s="7" t="s">
         <v>245</v>
       </c>
@@ -4531,11 +4841,11 @@
       <c r="I83" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="O83" s="2" t="s">
+      <c r="P83" s="2" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="84" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A84" s="7" t="s">
         <v>245</v>
       </c>
@@ -4554,11 +4864,11 @@
       <c r="I84" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="O84" s="2" t="s">
+      <c r="P84" s="2" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="85" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A85" s="7" t="s">
         <v>245</v>
       </c>
@@ -4577,11 +4887,11 @@
       <c r="I85" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="O85" s="2" t="s">
+      <c r="P85" s="2" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="86" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A86" s="7" t="s">
         <v>245</v>
       </c>
@@ -4600,11 +4910,11 @@
       <c r="I86" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="O86" s="2" t="s">
+      <c r="P86" s="2" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="87" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A87" s="7" t="s">
         <v>245</v>
       </c>
@@ -4626,11 +4936,11 @@
       <c r="I87" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q87" s="2" t="s">
+      <c r="R87" s="2" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="88" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A88" s="7" t="s">
         <v>245</v>
       </c>
@@ -4652,11 +4962,11 @@
       <c r="I88" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q88" s="2" t="s">
+      <c r="R88" s="2" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="89" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A89" s="7" t="s">
         <v>245</v>
       </c>
@@ -4678,11 +4988,11 @@
       <c r="I89" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q89" s="2" t="s">
+      <c r="R89" s="2" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="90" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A90" s="7" t="s">
         <v>245</v>
       </c>
@@ -4704,11 +5014,11 @@
       <c r="I90" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q90" s="2" t="s">
+      <c r="R90" s="2" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="91" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A91" s="7" t="s">
         <v>245</v>
       </c>
@@ -4730,11 +5040,11 @@
       <c r="I91" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q91" s="2" t="s">
+      <c r="R91" s="2" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="92" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A92" s="7" t="s">
         <v>245</v>
       </c>
@@ -4756,11 +5066,11 @@
       <c r="I92" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q92" s="2" t="s">
+      <c r="R92" s="2" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="93" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A93" s="7" t="s">
         <v>245</v>
       </c>
@@ -4782,11 +5092,11 @@
       <c r="I93" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q93" s="2" t="s">
+      <c r="R93" s="2" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="94" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A94" s="7" t="s">
         <v>245</v>
       </c>
@@ -4808,11 +5118,11 @@
       <c r="I94" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q94" s="2" t="s">
+      <c r="R94" s="2" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="95" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A95" s="7" t="s">
         <v>245</v>
       </c>
@@ -4834,11 +5144,11 @@
       <c r="I95" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q95" s="2" t="s">
+      <c r="R95" s="2" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="96" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A96" s="7" t="s">
         <v>245</v>
       </c>
@@ -4860,11 +5170,11 @@
       <c r="I96" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q96" s="2" t="s">
+      <c r="R96" s="2" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="97" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A97" s="7" t="s">
         <v>245</v>
       </c>
@@ -4886,11 +5196,11 @@
       <c r="I97" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q97" s="2" t="s">
+      <c r="R97" s="2" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="98" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A98" s="7" t="s">
         <v>245</v>
       </c>
@@ -4903,11 +5213,11 @@
       <c r="G98" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="Q98" s="2" t="s">
+      <c r="R98" s="2" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="99" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A99" s="7" t="s">
         <v>245</v>
       </c>
@@ -4917,11 +5227,11 @@
       <c r="G99" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="Q99" s="2" t="s">
+      <c r="R99" s="2" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="100" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A100" s="7" t="s">
         <v>245</v>
       </c>
@@ -4944,7 +5254,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="101" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A101" s="7" t="s">
         <v>245</v>
       </c>
@@ -4966,11 +5276,11 @@
       <c r="I101" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q101" s="2" t="s">
+      <c r="R101" s="2" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="102" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A102" s="7" t="s">
         <v>245</v>
       </c>
@@ -4992,11 +5302,11 @@
       <c r="I102" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q102" s="2" t="s">
+      <c r="R102" s="2" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="103" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A103" s="7" t="s">
         <v>245</v>
       </c>
@@ -5018,11 +5328,11 @@
       <c r="I103" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q103" s="2" t="s">
+      <c r="R103" s="2" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="104" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A104" s="7" t="s">
         <v>245</v>
       </c>
@@ -5044,11 +5354,11 @@
       <c r="I104" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="Q104" s="2" t="s">
+      <c r="R104" s="2" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="105" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A105" s="7" t="s">
         <v>245</v>
       </c>
@@ -5070,11 +5380,11 @@
       <c r="I105" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q105" s="2" t="s">
+      <c r="R105" s="2" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="106" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A106" s="7" t="s">
         <v>245</v>
       </c>
@@ -5096,11 +5406,11 @@
       <c r="I106" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q106" s="2" t="s">
+      <c r="R106" s="2" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="107" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A107" s="7" t="s">
         <v>245</v>
       </c>
@@ -5122,11 +5432,11 @@
       <c r="I107" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q107" s="2" t="s">
+      <c r="R107" s="2" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="108" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A108" s="7" t="s">
         <v>245</v>
       </c>
@@ -5148,11 +5458,11 @@
       <c r="I108" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q108" s="2" t="s">
+      <c r="R108" s="2" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="109" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A109" s="7" t="s">
         <v>245</v>
       </c>
@@ -5174,11 +5484,11 @@
       <c r="I109" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q109" s="2" t="s">
+      <c r="R109" s="2" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="110" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A110" s="7" t="s">
         <v>245</v>
       </c>
@@ -5200,11 +5510,11 @@
       <c r="I110" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q110" s="2" t="s">
+      <c r="R110" s="2" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="111" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A111" s="7" t="s">
         <v>245</v>
       </c>
@@ -5226,11 +5536,11 @@
       <c r="I111" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="Q111" s="2" t="s">
+      <c r="R111" s="2" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="112" spans="1:17" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:18" s="7" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A112" s="7" t="s">
         <v>245</v>
       </c>
@@ -5249,14 +5559,14 @@
       <c r="I112" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="P112" s="30" t="s">
-        <v>312</v>
-      </c>
       <c r="Q112" s="30" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="113" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+      <c r="R112" s="30" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="113" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A113" s="8" t="s">
         <v>323</v>
       </c>
@@ -5278,17 +5588,17 @@
       <c r="I113" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="O113" s="39" t="s">
+      <c r="P113" s="39" t="s">
         <v>324</v>
       </c>
-      <c r="P113" s="9" t="s">
+      <c r="Q113" s="9" t="s">
         <v>313</v>
       </c>
-      <c r="Q113" s="39" t="s">
+      <c r="R113" s="39" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="114" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A114" s="8" t="s">
         <v>323</v>
       </c>
@@ -5310,17 +5620,17 @@
       <c r="I114" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="O114" s="39" t="s">
+      <c r="P114" s="39" t="s">
         <v>325</v>
       </c>
-      <c r="P114" s="9" t="s">
+      <c r="Q114" s="9" t="s">
         <v>316</v>
       </c>
-      <c r="Q114" s="39" t="s">
+      <c r="R114" s="39" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="115" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A115" s="8" t="s">
         <v>323</v>
       </c>
@@ -5342,17 +5652,17 @@
       <c r="I115" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="O115" s="39" t="s">
+      <c r="P115" s="39" t="s">
         <v>326</v>
       </c>
-      <c r="P115" s="9" t="s">
+      <c r="Q115" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="Q115" s="39" t="s">
+      <c r="R115" s="39" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="116" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A116" s="8" t="s">
         <v>323</v>
       </c>
@@ -5374,14 +5684,14 @@
       <c r="I116" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="O116" s="39" t="s">
+      <c r="P116" s="39" t="s">
         <v>327</v>
       </c>
-      <c r="P116" s="9" t="s">
+      <c r="Q116" s="9" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="117" spans="1:17" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:18" s="8" customFormat="1" ht="32" x14ac:dyDescent="0.4">
       <c r="A117" s="8" t="s">
         <v>323</v>
       </c>
@@ -5403,14 +5713,14 @@
       <c r="I117" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="O117" s="39" t="s">
+      <c r="P117" s="39" t="s">
         <v>328</v>
       </c>
-      <c r="P117" s="9" t="s">
+      <c r="Q117" s="9" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="118" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A118" s="7" t="s">
         <v>333</v>
       </c>
@@ -5432,11 +5742,11 @@
       <c r="I118" s="7" t="s">
         <v>348</v>
       </c>
-      <c r="O118" s="7" t="s">
+      <c r="P118" s="7" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="119" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A119" s="7" t="s">
         <v>333</v>
       </c>
@@ -5455,11 +5765,11 @@
       <c r="I119" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="O119" s="7" t="s">
+      <c r="P119" s="7" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="120" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A120" s="7" t="s">
         <v>333</v>
       </c>
@@ -5478,11 +5788,11 @@
       <c r="I120" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="O120" s="7" t="s">
+      <c r="P120" s="7" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="121" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A121" s="7" t="s">
         <v>333</v>
       </c>
@@ -5501,11 +5811,11 @@
       <c r="I121" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="O121" s="7" t="s">
+      <c r="P121" s="7" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="122" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A122" s="7" t="s">
         <v>333</v>
       </c>
@@ -5524,11 +5834,11 @@
       <c r="I122" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="O122" s="7" t="s">
+      <c r="P122" s="7" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="123" spans="1:17" s="7" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:18" s="7" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A123" s="7" t="s">
         <v>333</v>
       </c>
@@ -5547,11 +5857,11 @@
       <c r="I123" s="7" t="s">
         <v>348</v>
       </c>
-      <c r="O123" s="7" t="s">
+      <c r="P123" s="7" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="124" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A124" s="7" t="s">
         <v>333</v>
       </c>
@@ -5570,11 +5880,11 @@
       <c r="I124" s="7" t="s">
         <v>349</v>
       </c>
-      <c r="O124" s="7" t="s">
+      <c r="P124" s="7" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="125" spans="1:17" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:18" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A125" s="8" t="s">
         <v>350</v>
       </c>
@@ -5596,11 +5906,11 @@
       <c r="I125" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O125" s="8" t="s">
+      <c r="P125" s="8" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="126" spans="1:17" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:18" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A126" s="8" t="s">
         <v>350</v>
       </c>
@@ -5619,11 +5929,11 @@
       <c r="I126" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O126" s="8" t="s">
+      <c r="P126" s="8" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="127" spans="1:17" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:18" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A127" s="8" t="s">
         <v>350</v>
       </c>
@@ -5642,11 +5952,11 @@
       <c r="I127" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O127" s="8" t="s">
+      <c r="P127" s="8" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="128" spans="1:17" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:18" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A128" s="8" t="s">
         <v>350</v>
       </c>
@@ -5665,11 +5975,11 @@
       <c r="I128" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O128" s="8" t="s">
+      <c r="P128" s="8" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="129" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A129" s="8" t="s">
         <v>350</v>
       </c>
@@ -5688,11 +5998,11 @@
       <c r="I129" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O129" s="8" t="s">
+      <c r="P129" s="8" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="130" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A130" s="8" t="s">
         <v>350</v>
       </c>
@@ -5711,11 +6021,11 @@
       <c r="I130" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O130" s="8" t="s">
+      <c r="P130" s="8" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="131" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A131" s="8" t="s">
         <v>350</v>
       </c>
@@ -5734,11 +6044,11 @@
       <c r="I131" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O131" s="8" t="s">
+      <c r="P131" s="8" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="132" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A132" s="8" t="s">
         <v>350</v>
       </c>
@@ -5757,11 +6067,11 @@
       <c r="I132" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O132" s="8" t="s">
+      <c r="P132" s="8" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="133" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A133" s="8" t="s">
         <v>350</v>
       </c>
@@ -5780,11 +6090,11 @@
       <c r="I133" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O133" s="8" t="s">
+      <c r="P133" s="8" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="134" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A134" s="8" t="s">
         <v>350</v>
       </c>
@@ -5803,11 +6113,11 @@
       <c r="I134" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O134" s="8" t="s">
+      <c r="P134" s="8" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="135" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A135" s="8" t="s">
         <v>350</v>
       </c>
@@ -5826,11 +6136,11 @@
       <c r="I135" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O135" s="8" t="s">
+      <c r="P135" s="8" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="136" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A136" s="8" t="s">
         <v>350</v>
       </c>
@@ -5849,11 +6159,11 @@
       <c r="I136" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O136" s="8" t="s">
+      <c r="P136" s="8" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="137" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A137" s="8" t="s">
         <v>350</v>
       </c>
@@ -5872,11 +6182,11 @@
       <c r="I137" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O137" s="8" t="s">
+      <c r="P137" s="8" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="138" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A138" s="8" t="s">
         <v>350</v>
       </c>
@@ -5895,11 +6205,11 @@
       <c r="I138" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O138" s="8" t="s">
+      <c r="P138" s="8" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="139" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A139" s="8" t="s">
         <v>350</v>
       </c>
@@ -5918,11 +6228,11 @@
       <c r="I139" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O139" s="8" t="s">
+      <c r="P139" s="8" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="140" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A140" s="8" t="s">
         <v>350</v>
       </c>
@@ -5941,11 +6251,11 @@
       <c r="I140" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O140" s="8" t="s">
+      <c r="P140" s="8" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="141" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A141" s="8" t="s">
         <v>350</v>
       </c>
@@ -5964,11 +6274,11 @@
       <c r="I141" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O141" s="8" t="s">
+      <c r="P141" s="8" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="142" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A142" s="8" t="s">
         <v>350</v>
       </c>
@@ -5987,11 +6297,11 @@
       <c r="I142" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O142" s="8" t="s">
+      <c r="P142" s="8" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="143" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A143" s="8" t="s">
         <v>350</v>
       </c>
@@ -6010,11 +6320,11 @@
       <c r="I143" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O143" s="8" t="s">
+      <c r="P143" s="8" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="144" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A144" s="8" t="s">
         <v>350</v>
       </c>
@@ -6033,11 +6343,11 @@
       <c r="I144" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O144" s="8" t="s">
+      <c r="P144" s="8" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="145" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A145" s="8" t="s">
         <v>350</v>
       </c>
@@ -6056,11 +6366,11 @@
       <c r="I145" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O145" s="8" t="s">
+      <c r="P145" s="8" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="146" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A146" s="8" t="s">
         <v>350</v>
       </c>
@@ -6079,11 +6389,11 @@
       <c r="I146" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O146" s="8" t="s">
+      <c r="P146" s="8" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="147" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A147" s="8" t="s">
         <v>350</v>
       </c>
@@ -6102,11 +6412,11 @@
       <c r="I147" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O147" s="8" t="s">
+      <c r="P147" s="8" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="148" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A148" s="8" t="s">
         <v>350</v>
       </c>
@@ -6125,11 +6435,11 @@
       <c r="I148" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O148" s="8" t="s">
+      <c r="P148" s="8" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="149" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A149" s="8" t="s">
         <v>350</v>
       </c>
@@ -6148,11 +6458,11 @@
       <c r="I149" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O149" s="8" t="s">
+      <c r="P149" s="8" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="150" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A150" s="8" t="s">
         <v>350</v>
       </c>
@@ -6171,11 +6481,11 @@
       <c r="I150" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O150" s="8" t="s">
+      <c r="P150" s="8" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="151" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A151" s="8" t="s">
         <v>350</v>
       </c>
@@ -6194,11 +6504,11 @@
       <c r="I151" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O151" s="8" t="s">
+      <c r="P151" s="8" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="152" spans="1:15" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:16" s="8" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A152" s="8" t="s">
         <v>350</v>
       </c>
@@ -6217,11 +6527,11 @@
       <c r="I152" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O152" s="8" t="s">
+      <c r="P152" s="8" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="153" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A153" s="8" t="s">
         <v>350</v>
       </c>
@@ -6240,11 +6550,11 @@
       <c r="I153" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O153" s="8" t="s">
+      <c r="P153" s="8" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="154" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A154" s="8" t="s">
         <v>350</v>
       </c>
@@ -6263,11 +6573,11 @@
       <c r="I154" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O154" s="8" t="s">
+      <c r="P154" s="8" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="155" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A155" s="8" t="s">
         <v>350</v>
       </c>
@@ -6286,11 +6596,11 @@
       <c r="I155" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="O155" s="8" t="s">
+      <c r="P155" s="8" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="156" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A156" s="8" t="s">
         <v>350</v>
       </c>
@@ -6309,11 +6619,11 @@
       <c r="I156" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O156" s="8" t="s">
+      <c r="P156" s="8" t="s">
         <v>440</v>
       </c>
     </row>
-    <row r="157" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A157" s="8" t="s">
         <v>350</v>
       </c>
@@ -6332,11 +6642,11 @@
       <c r="I157" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O157" s="8" t="s">
+      <c r="P157" s="8" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="158" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A158" s="8" t="s">
         <v>350</v>
       </c>
@@ -6355,11 +6665,11 @@
       <c r="I158" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O158" s="8" t="s">
+      <c r="P158" s="8" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="159" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A159" s="8" t="s">
         <v>350</v>
       </c>
@@ -6378,11 +6688,11 @@
       <c r="I159" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O159" s="8" t="s">
+      <c r="P159" s="8" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="160" spans="1:15" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A160" s="8" t="s">
         <v>350</v>
       </c>
@@ -6401,11 +6711,11 @@
       <c r="I160" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O160" s="8" t="s">
+      <c r="P160" s="8" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="161" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A161" s="8" t="s">
         <v>350</v>
       </c>
@@ -6424,11 +6734,11 @@
       <c r="I161" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O161" s="8" t="s">
+      <c r="P161" s="8" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="162" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A162" s="8" t="s">
         <v>350</v>
       </c>
@@ -6447,11 +6757,11 @@
       <c r="I162" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="O162" s="8" t="s">
+      <c r="P162" s="8" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="163" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A163" s="7" t="s">
         <v>350</v>
       </c>
@@ -6476,11 +6786,11 @@
       <c r="J163" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P163" s="7" t="s">
+      <c r="Q163" s="7" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="164" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A164" s="7" t="s">
         <v>350</v>
       </c>
@@ -6502,11 +6812,11 @@
       <c r="J164" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P164" s="7" t="s">
+      <c r="Q164" s="7" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="165" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A165" s="7" t="s">
         <v>350</v>
       </c>
@@ -6528,11 +6838,11 @@
       <c r="J165" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P165" s="7" t="s">
+      <c r="Q165" s="7" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="166" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A166" s="7" t="s">
         <v>350</v>
       </c>
@@ -6554,11 +6864,11 @@
       <c r="J166" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P166" s="7" t="s">
+      <c r="Q166" s="7" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="167" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A167" s="7" t="s">
         <v>350</v>
       </c>
@@ -6580,11 +6890,11 @@
       <c r="J167" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P167" s="7" t="s">
+      <c r="Q167" s="7" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="168" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A168" s="7" t="s">
         <v>350</v>
       </c>
@@ -6606,11 +6916,11 @@
       <c r="J168" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P168" s="7" t="s">
+      <c r="Q168" s="7" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="169" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A169" s="7" t="s">
         <v>350</v>
       </c>
@@ -6632,11 +6942,11 @@
       <c r="J169" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P169" s="7" t="s">
+      <c r="Q169" s="7" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="170" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A170" s="7" t="s">
         <v>350</v>
       </c>
@@ -6658,11 +6968,11 @@
       <c r="J170" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P170" s="7" t="s">
+      <c r="Q170" s="7" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="171" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A171" s="7" t="s">
         <v>350</v>
       </c>
@@ -6684,11 +6994,11 @@
       <c r="J171" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P171" s="7" t="s">
+      <c r="Q171" s="7" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="172" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A172" s="7" t="s">
         <v>350</v>
       </c>
@@ -6710,11 +7020,11 @@
       <c r="J172" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P172" s="7" t="s">
+      <c r="Q172" s="7" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="173" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A173" s="7" t="s">
         <v>350</v>
       </c>
@@ -6736,11 +7046,11 @@
       <c r="J173" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P173" s="7" t="s">
+      <c r="Q173" s="7" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="174" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:18" s="7" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A174" s="7" t="s">
         <v>350</v>
       </c>
@@ -6762,11 +7072,11 @@
       <c r="J174" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="P174" s="7" t="s">
+      <c r="Q174" s="7" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="175" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A175" s="25" t="s">
         <v>454</v>
       </c>
@@ -6791,11 +7101,11 @@
       <c r="J175" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q175" s="24" t="s">
+      <c r="R175" s="24" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="176" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A176" s="25" t="s">
         <v>459</v>
       </c>
@@ -6817,11 +7127,11 @@
       <c r="J176" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q176" s="25" t="s">
+      <c r="R176" s="25" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="177" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A177" s="25" t="s">
         <v>461</v>
       </c>
@@ -6843,11 +7153,11 @@
       <c r="J177" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q177" s="25" t="s">
+      <c r="R177" s="25" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="178" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A178" s="25" t="s">
         <v>461</v>
       </c>
@@ -6872,11 +7182,11 @@
       <c r="J178" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q178" s="25" t="s">
+      <c r="R178" s="25" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="179" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A179" s="25" t="s">
         <v>461</v>
       </c>
@@ -6901,11 +7211,11 @@
       <c r="J179" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q179" s="25" t="s">
+      <c r="R179" s="25" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="180" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A180" s="25" t="s">
         <v>466</v>
       </c>
@@ -6930,11 +7240,11 @@
       <c r="J180" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q180" s="25" t="s">
+      <c r="R180" s="25" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="181" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A181" s="25" t="s">
         <v>471</v>
       </c>
@@ -6956,11 +7266,11 @@
       <c r="J181" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q181" s="25" t="s">
+      <c r="R181" s="25" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="182" spans="1:17" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:18" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A182" s="25" t="s">
         <v>474</v>
       </c>
@@ -6982,11 +7292,11 @@
       <c r="J182" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q182" s="25" t="s">
+      <c r="R182" s="25" t="s">
         <v>476</v>
       </c>
     </row>
-    <row r="183" spans="1:17" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:18" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A183" s="25" t="s">
         <v>474</v>
       </c>
@@ -7008,11 +7318,11 @@
       <c r="J183" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q183" s="25" t="s">
+      <c r="R183" s="25" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="184" spans="1:17" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:18" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A184" s="25" t="s">
         <v>474</v>
       </c>
@@ -7034,11 +7344,11 @@
       <c r="J184" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q184" s="42" t="s">
+      <c r="R184" s="42" t="s">
         <v>480</v>
       </c>
     </row>
-    <row r="185" spans="1:17" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:18" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A185" s="25" t="s">
         <v>481</v>
       </c>
@@ -7060,11 +7370,11 @@
       <c r="J185" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q185" s="24" t="s">
+      <c r="R185" s="24" t="s">
         <v>483</v>
       </c>
     </row>
-    <row r="186" spans="1:17" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:18" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A186" s="25" t="s">
         <v>481</v>
       </c>
@@ -7086,11 +7396,11 @@
       <c r="J186" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q186" s="24" t="s">
+      <c r="R186" s="24" t="s">
         <v>486</v>
       </c>
     </row>
-    <row r="187" spans="1:17" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:18" s="25" customFormat="1" ht="24" x14ac:dyDescent="0.3">
       <c r="A187" s="25" t="s">
         <v>481</v>
       </c>
@@ -7112,11 +7422,11 @@
       <c r="J187" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q187" s="24" t="s">
+      <c r="R187" s="24" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="188" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A188" s="25" t="s">
         <v>481</v>
       </c>
@@ -7138,11 +7448,11 @@
       <c r="J188" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q188" s="25" t="s">
+      <c r="R188" s="25" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="189" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A189" s="25" t="s">
         <v>481</v>
       </c>
@@ -7164,11 +7474,11 @@
       <c r="J189" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q189" s="25" t="s">
+      <c r="R189" s="25" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="190" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A190" s="25" t="s">
         <v>481</v>
       </c>
@@ -7190,11 +7500,11 @@
       <c r="J190" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q190" s="25" t="s">
+      <c r="R190" s="25" t="s">
         <v>499</v>
       </c>
     </row>
-    <row r="191" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A191" s="25" t="s">
         <v>481</v>
       </c>
@@ -7216,11 +7526,11 @@
       <c r="J191" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q191" s="25" t="s">
+      <c r="R191" s="25" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="192" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A192" s="25" t="s">
         <v>481</v>
       </c>
@@ -7242,11 +7552,11 @@
       <c r="J192" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q192" s="25" t="s">
+      <c r="R192" s="25" t="s">
         <v>501</v>
       </c>
     </row>
-    <row r="193" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A193" s="25" t="s">
         <v>481</v>
       </c>
@@ -7268,11 +7578,11 @@
       <c r="J193" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q193" s="25" t="s">
+      <c r="R193" s="25" t="s">
         <v>502</v>
       </c>
     </row>
-    <row r="194" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A194" s="25" t="s">
         <v>481</v>
       </c>
@@ -7294,11 +7604,11 @@
       <c r="J194" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q194" s="25" t="s">
+      <c r="R194" s="25" t="s">
         <v>503</v>
       </c>
     </row>
-    <row r="195" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A195" s="25" t="s">
         <v>481</v>
       </c>
@@ -7320,11 +7630,11 @@
       <c r="J195" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q195" s="25" t="s">
+      <c r="R195" s="25" t="s">
         <v>504</v>
       </c>
     </row>
-    <row r="196" spans="1:17" s="25" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:18" s="25" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A196" s="25" t="s">
         <v>481</v>
       </c>
@@ -7346,11 +7656,11 @@
       <c r="J196" s="25" t="s">
         <v>456</v>
       </c>
-      <c r="Q196" s="25" t="s">
+      <c r="R196" s="25" t="s">
         <v>505</v>
       </c>
     </row>
-    <row r="197" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A197" s="8" t="s">
         <v>508</v>
       </c>
@@ -7375,11 +7685,11 @@
       <c r="J197" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P197" s="44" t="s">
+      <c r="Q197" s="44" t="s">
         <v>511</v>
       </c>
     </row>
-    <row r="198" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A198" s="8" t="s">
         <v>508</v>
       </c>
@@ -7401,11 +7711,11 @@
       <c r="J198" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P198" s="44" t="s">
+      <c r="Q198" s="44" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="199" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A199" s="8" t="s">
         <v>508</v>
       </c>
@@ -7427,11 +7737,11 @@
       <c r="J199" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P199" s="44" t="s">
+      <c r="Q199" s="44" t="s">
         <v>513</v>
       </c>
     </row>
-    <row r="200" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A200" s="8" t="s">
         <v>508</v>
       </c>
@@ -7453,11 +7763,11 @@
       <c r="J200" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P200" s="44" t="s">
+      <c r="Q200" s="44" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="201" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A201" s="8" t="s">
         <v>508</v>
       </c>
@@ -7479,11 +7789,11 @@
       <c r="J201" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P201" s="44" t="s">
+      <c r="Q201" s="44" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="202" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A202" s="8" t="s">
         <v>508</v>
       </c>
@@ -7505,11 +7815,11 @@
       <c r="J202" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P202" s="44" t="s">
+      <c r="Q202" s="44" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="203" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A203" s="8" t="s">
         <v>508</v>
       </c>
@@ -7531,11 +7841,11 @@
       <c r="J203" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P203" s="44" t="s">
+      <c r="Q203" s="44" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="204" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A204" s="8" t="s">
         <v>508</v>
       </c>
@@ -7557,11 +7867,11 @@
       <c r="J204" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P204" s="44" t="s">
+      <c r="Q204" s="44" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="205" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A205" s="8" t="s">
         <v>508</v>
       </c>
@@ -7583,11 +7893,11 @@
       <c r="J205" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P205" s="44" t="s">
+      <c r="Q205" s="44" t="s">
         <v>519</v>
       </c>
     </row>
-    <row r="206" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A206" s="8" t="s">
         <v>508</v>
       </c>
@@ -7609,11 +7919,11 @@
       <c r="J206" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P206" s="44" t="s">
+      <c r="Q206" s="44" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="207" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A207" s="8" t="s">
         <v>508</v>
       </c>
@@ -7635,11 +7945,11 @@
       <c r="J207" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P207" s="44" t="s">
+      <c r="Q207" s="44" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="208" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:18" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A208" s="8" t="s">
         <v>508</v>
       </c>
@@ -7661,11 +7971,11 @@
       <c r="J208" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P208" s="44" t="s">
+      <c r="Q208" s="44" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="209" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A209" s="8" t="s">
         <v>508</v>
       </c>
@@ -7687,11 +7997,11 @@
       <c r="J209" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P209" s="44" t="s">
+      <c r="Q209" s="44" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="210" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A210" s="8" t="s">
         <v>508</v>
       </c>
@@ -7713,11 +8023,11 @@
       <c r="J210" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P210" s="44" t="s">
+      <c r="Q210" s="44" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="211" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A211" s="8" t="s">
         <v>508</v>
       </c>
@@ -7739,8 +8049,695 @@
       <c r="J211" s="8" t="s">
         <v>457</v>
       </c>
-      <c r="P211" s="44" t="s">
+      <c r="Q211" s="44" t="s">
         <v>525</v>
+      </c>
+    </row>
+    <row r="214" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A214" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="C214" s="62" t="s">
+        <v>619</v>
+      </c>
+      <c r="D214" s="46" t="s">
+        <v>547</v>
+      </c>
+      <c r="E214" s="31">
+        <v>14.49493</v>
+      </c>
+      <c r="F214" s="31">
+        <v>101.9314</v>
+      </c>
+      <c r="G214" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="I214" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="L214" s="47" t="s">
+        <v>545</v>
+      </c>
+      <c r="P214" s="48" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="215" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A215" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="D215" s="46" t="s">
+        <v>548</v>
+      </c>
+      <c r="E215" s="31">
+        <v>14.49493</v>
+      </c>
+      <c r="F215" s="31">
+        <v>101.9314</v>
+      </c>
+      <c r="G215" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="I215" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="L215" s="47" t="s">
+        <v>546</v>
+      </c>
+      <c r="P215" s="48" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="216" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A216" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="D216" s="49" t="s">
+        <v>549</v>
+      </c>
+      <c r="E216" s="31">
+        <v>12.52819</v>
+      </c>
+      <c r="F216" s="31">
+        <v>102.1828</v>
+      </c>
+      <c r="G216" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="I216" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="P216" s="49" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="217" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A217" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="D217" s="49" t="s">
+        <v>551</v>
+      </c>
+      <c r="E217" s="31">
+        <v>18.878589999999999</v>
+      </c>
+      <c r="F217" s="31">
+        <v>101.1906</v>
+      </c>
+      <c r="G217" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="I217" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="L217" s="47" t="s">
+        <v>555</v>
+      </c>
+      <c r="P217" s="50" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="218" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A218" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="D218" s="49" t="s">
+        <v>552</v>
+      </c>
+      <c r="E218" s="31">
+        <v>18.878589999999999</v>
+      </c>
+      <c r="F218" s="31">
+        <v>101.1906</v>
+      </c>
+      <c r="G218" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="I218" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="L218" s="47" t="s">
+        <v>556</v>
+      </c>
+      <c r="P218" s="50" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="219" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A219" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="D219" s="49" t="s">
+        <v>557</v>
+      </c>
+      <c r="E219" s="31">
+        <v>17.976980000000001</v>
+      </c>
+      <c r="F219" s="31">
+        <v>102.6126</v>
+      </c>
+      <c r="G219" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="I219" s="31" t="s">
+        <v>565</v>
+      </c>
+      <c r="P219" s="49" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="220" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A220" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="D220" s="49" t="s">
+        <v>559</v>
+      </c>
+      <c r="E220" s="31">
+        <v>17.898790000000002</v>
+      </c>
+      <c r="F220" s="31">
+        <v>105.31319999999999</v>
+      </c>
+      <c r="G220" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="I220" s="31" t="s">
+        <v>565</v>
+      </c>
+      <c r="L220" s="46" t="s">
+        <v>561</v>
+      </c>
+      <c r="P220" s="48" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="221" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A221" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="D221" s="49" t="s">
+        <v>562</v>
+      </c>
+      <c r="E221" s="31">
+        <v>17.377210000000002</v>
+      </c>
+      <c r="F221" s="31">
+        <v>106.148</v>
+      </c>
+      <c r="G221" s="31" t="s">
+        <v>564</v>
+      </c>
+      <c r="I221" s="31" t="s">
+        <v>565</v>
+      </c>
+      <c r="P221" s="50" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="222" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A222" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="D222" s="46" t="s">
+        <v>566</v>
+      </c>
+      <c r="E222" s="31">
+        <v>16.384139999999999</v>
+      </c>
+      <c r="F222" s="31">
+        <v>107.4439</v>
+      </c>
+      <c r="G222" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="I222" s="31" t="s">
+        <v>565</v>
+      </c>
+      <c r="P222" s="48" t="s">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="223" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A223" s="31" t="s">
+        <v>541</v>
+      </c>
+      <c r="D223" s="46" t="s">
+        <v>567</v>
+      </c>
+      <c r="E223" s="31">
+        <v>16.384139999999999</v>
+      </c>
+      <c r="F223" s="31">
+        <v>107.4439</v>
+      </c>
+      <c r="G223" s="31" t="s">
+        <v>185</v>
+      </c>
+      <c r="I223" s="31" t="s">
+        <v>565</v>
+      </c>
+      <c r="P223" s="48" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="224" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A224" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="C224" s="62" t="s">
+        <v>619</v>
+      </c>
+      <c r="D224" s="51" t="s">
+        <v>570</v>
+      </c>
+      <c r="E224" s="8">
+        <v>24.428329999999999</v>
+      </c>
+      <c r="F224" s="8">
+        <v>99.283929999999998</v>
+      </c>
+      <c r="G224" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I224" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L224" s="52" t="s">
+        <v>572</v>
+      </c>
+      <c r="P224" s="53" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="225" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A225" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D225" s="54" t="s">
+        <v>575</v>
+      </c>
+      <c r="E225" s="8">
+        <v>24.428329999999999</v>
+      </c>
+      <c r="F225" s="8">
+        <v>99.283929999999998</v>
+      </c>
+      <c r="G225" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I225" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L225" s="52" t="s">
+        <v>574</v>
+      </c>
+      <c r="P225" s="53" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="226" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A226" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D226" s="54" t="s">
+        <v>578</v>
+      </c>
+      <c r="E226" s="8">
+        <v>25.077100000000002</v>
+      </c>
+      <c r="F226" s="8">
+        <v>99.192660000000004</v>
+      </c>
+      <c r="G226" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I226" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L226" s="52" t="s">
+        <v>577</v>
+      </c>
+      <c r="P226" s="53" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="227" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A227" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D227" s="54" t="s">
+        <v>581</v>
+      </c>
+      <c r="E227" s="8">
+        <v>25.077100000000002</v>
+      </c>
+      <c r="F227" s="8">
+        <v>99.192660000000004</v>
+      </c>
+      <c r="G227" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I227" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L227" s="51" t="s">
+        <v>580</v>
+      </c>
+      <c r="P227" s="53" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="228" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A228" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D228" s="51" t="s">
+        <v>586</v>
+      </c>
+      <c r="E228" s="8">
+        <v>24.048999999999999</v>
+      </c>
+      <c r="F228" s="8">
+        <v>100.5162</v>
+      </c>
+      <c r="G228" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I228" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="L228" s="52" t="s">
+        <v>583</v>
+      </c>
+      <c r="P228" s="53" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="229" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A229" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D229" s="51" t="s">
+        <v>587</v>
+      </c>
+      <c r="E229" s="8">
+        <v>24.048999999999999</v>
+      </c>
+      <c r="F229" s="8">
+        <v>100.5162</v>
+      </c>
+      <c r="G229" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I229" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="L229" s="52" t="s">
+        <v>585</v>
+      </c>
+      <c r="P229" s="53" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="230" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A230" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D230" s="54" t="s">
+        <v>588</v>
+      </c>
+      <c r="E230" s="8">
+        <v>24.374140000000001</v>
+      </c>
+      <c r="F230" s="8">
+        <v>100.24290000000001</v>
+      </c>
+      <c r="G230" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I230" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="P230" s="55" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="231" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A231" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D231" s="51" t="s">
+        <v>590</v>
+      </c>
+      <c r="E231" s="8">
+        <v>21.978380000000001</v>
+      </c>
+      <c r="F231" s="8">
+        <v>101.46939999999999</v>
+      </c>
+      <c r="G231" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I231" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="L231" s="52" t="s">
+        <v>593</v>
+      </c>
+      <c r="P231" s="53" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="232" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A232" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D232" s="51" t="s">
+        <v>591</v>
+      </c>
+      <c r="E232" s="8">
+        <v>21.978380000000001</v>
+      </c>
+      <c r="F232" s="8">
+        <v>101.46939999999999</v>
+      </c>
+      <c r="G232" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I232" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="L232" s="52" t="s">
+        <v>595</v>
+      </c>
+      <c r="P232" s="53" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="233" spans="1:16" s="8" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A233" s="8" t="s">
+        <v>541</v>
+      </c>
+      <c r="D233" s="54" t="s">
+        <v>596</v>
+      </c>
+      <c r="E233" s="8">
+        <v>22.188510000000001</v>
+      </c>
+      <c r="F233" s="8">
+        <v>101.55070000000001</v>
+      </c>
+      <c r="G233" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="I233" s="8" t="s">
+        <v>565</v>
+      </c>
+      <c r="L233" s="51" t="s">
+        <v>598</v>
+      </c>
+      <c r="P233" s="53" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="234" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A234" s="27" t="s">
+        <v>599</v>
+      </c>
+      <c r="C234" s="62" t="s">
+        <v>619</v>
+      </c>
+      <c r="D234" s="56" t="s">
+        <v>600</v>
+      </c>
+      <c r="E234" s="27">
+        <v>26.2424</v>
+      </c>
+      <c r="F234" s="27">
+        <v>105.9449</v>
+      </c>
+      <c r="G234" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="I234" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="L234" s="57" t="s">
+        <v>602</v>
+      </c>
+      <c r="P234" s="58" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="235" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A235" s="27" t="s">
+        <v>599</v>
+      </c>
+      <c r="D235" s="56" t="s">
+        <v>603</v>
+      </c>
+      <c r="E235" s="27">
+        <v>23.658339999999999</v>
+      </c>
+      <c r="F235" s="27">
+        <v>103.34269999999999</v>
+      </c>
+      <c r="G235" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="I235" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="P235" s="59" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="236" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A236" s="27" t="s">
+        <v>599</v>
+      </c>
+      <c r="D236" s="60" t="s">
+        <v>605</v>
+      </c>
+      <c r="E236" s="27">
+        <v>22.534490000000002</v>
+      </c>
+      <c r="F236" s="27">
+        <v>105.0814</v>
+      </c>
+      <c r="G236" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="I236" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="L236" s="60" t="s">
+        <v>608</v>
+      </c>
+      <c r="P236" s="58" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="237" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A237" s="27" t="s">
+        <v>599</v>
+      </c>
+      <c r="D237" s="61" t="s">
+        <v>606</v>
+      </c>
+      <c r="E237" s="27">
+        <v>22.534490000000002</v>
+      </c>
+      <c r="F237" s="27">
+        <v>105.0814</v>
+      </c>
+      <c r="G237" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="I237" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="L237" s="57" t="s">
+        <v>610</v>
+      </c>
+      <c r="P237" s="58" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="238" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A238" s="27" t="s">
+        <v>599</v>
+      </c>
+      <c r="D238" s="56" t="s">
+        <v>611</v>
+      </c>
+      <c r="E238" s="27">
+        <v>22.007110000000001</v>
+      </c>
+      <c r="F238" s="27">
+        <v>105.8648</v>
+      </c>
+      <c r="G238" s="27" t="s">
+        <v>564</v>
+      </c>
+      <c r="I238" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="L238" s="57" t="s">
+        <v>615</v>
+      </c>
+      <c r="P238" s="58" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="239" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A239" s="27" t="s">
+        <v>599</v>
+      </c>
+      <c r="D239" s="61" t="s">
+        <v>612</v>
+      </c>
+      <c r="E239" s="27">
+        <v>22.007110000000001</v>
+      </c>
+      <c r="F239" s="27">
+        <v>105.8648</v>
+      </c>
+      <c r="G239" s="27" t="s">
+        <v>564</v>
+      </c>
+      <c r="I239" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="L239" s="57" t="s">
+        <v>617</v>
+      </c>
+      <c r="P239" s="58" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="240" spans="1:16" s="27" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A240" s="27" t="s">
+        <v>599</v>
+      </c>
+      <c r="D240" s="56" t="s">
+        <v>613</v>
+      </c>
+      <c r="E240" s="27">
+        <v>20.79973</v>
+      </c>
+      <c r="F240" s="27">
+        <v>106.9965</v>
+      </c>
+      <c r="G240" s="27" t="s">
+        <v>185</v>
+      </c>
+      <c r="I240" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="L240" s="59" t="s">
+        <v>618</v>
       </c>
     </row>
   </sheetData>
@@ -7757,6 +8754,9 @@
     <hyperlink ref="C179" r:id="rId9" display="https://doi.org/10.11646/zootaxa.4577.2.3" xr:uid="{EEB39083-DC07-6A4C-88DB-FEBFE4D307C2}"/>
     <hyperlink ref="C175" r:id="rId10" display="https://doi.org/10.7717/peerj.5575" xr:uid="{C90873C0-4263-0A41-A7E6-5314E79D0BEA}"/>
     <hyperlink ref="C197" r:id="rId11" tooltip="Persistent link using digital object identifier" xr:uid="{11E1C3B7-06EB-EA41-924E-8E5372B7B084}"/>
+    <hyperlink ref="C214" r:id="rId12" display="https://doi.org/10.1093/cz/zow042" xr:uid="{011D2AF8-C440-C545-A411-7934FC60DD9F}"/>
+    <hyperlink ref="C224" r:id="rId13" display="https://doi.org/10.1093/cz/zow042" xr:uid="{29808DD5-C151-894C-A4D3-26BEC910652A}"/>
+    <hyperlink ref="C234" r:id="rId14" display="https://doi.org/10.1093/cz/zow042" xr:uid="{5ACB5E97-6E77-1B4D-AD39-0726A7BEAB56}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added readme to mekong and red ecoevolity directories.
</commit_message>
<xml_diff>
--- a/Alignments_to_make.xlsx
+++ b/Alignments_to_make.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://byu-my.sharepoint.com/personal/rklaback_byu_edu/Documents/KlabackaLab/Research/SEA-riverine-barrier-popgen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1084" documentId="8_{8806978C-AB6D-854E-872D-B0339ADE4273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D4B15D8-E127-7849-9377-F9017EF4E8E4}"/>
+  <xr:revisionPtr revIDLastSave="1085" documentId="8_{8806978C-AB6D-854E-872D-B0339ADE4273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A05A342-5671-A849-8824-029F5E73C988}"/>
   <bookViews>
     <workbookView xWindow="9040" yWindow="660" windowWidth="21200" windowHeight="17300" xr2:uid="{A3120B5E-B713-6F49-8845-F185AE497150}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1427" uniqueCount="622">
   <si>
     <t>Species</t>
   </si>
@@ -1941,6 +1941,9 @@
   </si>
   <si>
     <t>Eutropis multifasciataUT</t>
+  </si>
+  <si>
+    <t>Trimer</t>
   </si>
 </sst>
 </file>
@@ -7774,6 +7777,9 @@
       <c r="A201" s="8" t="s">
         <v>508</v>
       </c>
+      <c r="B201" s="8" t="s">
+        <v>621</v>
+      </c>
       <c r="D201" s="45" t="s">
         <v>529</v>
       </c>

</xml_diff>